<commit_message>
docs+template: v2 team-scramble sheet template and runbook
</commit_message>
<xml_diff>
--- a/tools/gfy-template.xlsx
+++ b/tools/gfy-template.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,7 +486,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>36 holes, stroke</t>
+          <t>2-day scramble</t>
         </is>
       </c>
     </row>
@@ -535,6 +535,30 @@
       <c r="B9" t="inlineStr">
         <is>
           <t>gross</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>deposit_amount</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>payment_handle</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Venmo @gfy-duck</t>
         </is>
       </c>
     </row>
@@ -765,7 +789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -781,17 +805,32 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>since</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>handicap</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>deposit</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>paid_date</t>
         </is>
       </c>
     </row>
@@ -804,19 +843,28 @@
           <t>Duck</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Duck</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2019</v>
+      </c>
+      <c r="E2" t="n">
         <v>8</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>In</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -827,15 +875,28 @@
           <t>Hammer</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>12</v>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Duck</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2019</v>
+      </c>
+      <c r="E3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>In</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -846,15 +907,116 @@
           <t>Sully</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sully</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E4" t="n">
         <v>15</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Maybe</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>In</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tank</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Sully</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E5" t="n">
+        <v>20</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>In</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Tex</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Tex</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2019</v>
+      </c>
+      <c r="E6" t="n">
+        <v>18</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>In</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Duck</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -878,7 +1040,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>team</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -1050,7 +1212,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hammer</t>
+          <t>Sully</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -1117,7 +1279,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Sully</t>
+          <t>Tex</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1358,7 +1520,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Duck · Hammer · Sully</t>
+          <t>Duck · Hammer</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1545,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Moose · Tex</t>
+          <t>Sully · Tank</t>
         </is>
       </c>
     </row>
@@ -1434,7 +1596,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>team</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -1449,7 +1611,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>buyback</t>
+          <t>collected</t>
         </is>
       </c>
     </row>
@@ -1470,8 +1632,10 @@
       <c r="D2" t="n">
         <v>120</v>
       </c>
-      <c r="E2" t="n">
-        <v>50</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -1480,18 +1644,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hammer</t>
+          <t>Sully</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sully</t>
+          <t>Duck</t>
         </is>
       </c>
       <c r="D3" t="n">
         <v>100</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1499,19 +1667,21 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Moose</t>
+          <t>Tex</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Duck</t>
+          <t>Sully</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>80</v>
-      </c>
-      <c r="E4" t="n">
-        <v>25</v>
+        <v>90</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1636,7 +1806,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1825,11 @@
       <c r="D3" t="n">
         <v>40</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1672,7 +1846,11 @@
       <c r="D4" t="n">
         <v>0</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: invites funnel — outreach tracking on the next-year board (emails never render)
</commit_message>
<xml_diff>
--- a/tools/gfy-template.xlsx
+++ b/tools/gfy-template.xlsx
@@ -18,6 +18,7 @@
     <sheet name="Ledger" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Champions" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Shame" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Invites" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -719,6 +720,134 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>invited</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>responded</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Sully</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>sully@example.com</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Tex</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>tex@example.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>bear@example.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>out</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: v2.2 wave 1 — hardened anchors/dates/funnel privacy, stale-board live-bug fix, derived views, seasonal nav
</commit_message>
<xml_diff>
--- a/tools/gfy-template.xlsx
+++ b/tools/gfy-template.xlsx
@@ -726,7 +726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -742,20 +742,15 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>invited</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>invited</t>
+          <t>responded</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>responded</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -772,7 +767,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>sully@example.com</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -780,12 +775,7 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -798,20 +788,15 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>tex@example.com</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -824,7 +809,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>bear@example.com</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -833,11 +818,6 @@
         </is>
       </c>
       <c r="E4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
         <is>
           <t>out</t>
         </is>

</xml_diff>

<commit_message>
feat: v2.2 wave 2 — rooms, would-pay, committed-only owing, review-fix closure
</commit_message>
<xml_diff>
--- a/tools/gfy-template.xlsx
+++ b/tools/gfy-template.xlsx
@@ -19,6 +19,7 @@
     <sheet name="Champions" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Shame" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Invites" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Rooms" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -828,6 +829,122 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>property</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>room</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bear Creek Lodge</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Duck</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bear Creek Lodge</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Hammer</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Bear Creek Lodge</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sully</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bear Creek Lodge</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>guest:Pat</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: courseYards() + real MeadowCreek white-tee course data in template (C-REAL)
</commit_message>
<xml_diff>
--- a/tools/gfy-template.xlsx
+++ b/tools/gfy-template.xlsx
@@ -951,7 +951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -979,7 +979,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>385</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3">
@@ -987,10 +987,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" t="n">
-        <v>410</v>
+        <v>469</v>
       </c>
     </row>
     <row r="4">
@@ -998,10 +998,175 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
         <v>3</v>
       </c>
-      <c r="C4" t="n">
-        <v>175</v>
+      <c r="C5" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" t="n">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" t="n">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" t="n">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" t="n">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" t="n">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" t="n">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" t="n">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" t="n">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="n">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" t="n">
+        <v>533</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: P-SHOTGUN — optional Pairings start-hole column (additive, display-only)
</commit_message>
<xml_diff>
--- a/tools/gfy-template.xlsx
+++ b/tools/gfy-template.xlsx
@@ -1860,7 +1860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1889,6 +1889,11 @@
           <t>players</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1914,6 +1919,9 @@
           <t>Duck · Hammer</t>
         </is>
       </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1939,6 +1947,9 @@
           <t>Sully · Tank</t>
         </is>
       </c>
+      <c r="F3" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1964,6 +1975,7 @@
           <t>Leaders out last</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: N-FULLNAMES convention + §15 template columns (place/players/strengths) + draft docs
</commit_message>
<xml_diff>
--- a/tools/gfy-template.xlsx
+++ b/tools/gfy-template.xlsx
@@ -575,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,6 +594,16 @@
           <t>score</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>players</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -609,36 +619,92 @@
           <t>151 (+7)</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Duck · Hammer · Sully · Tank</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hammer</t>
+          <t>Tex</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>149 (+5)</t>
+          <t>153 (+9)</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Tex · Sock · Bear · Crash</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Moose</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>155 (+11)</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Moose · Ghost · Blade · Zeke</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hammer</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>149 (+5)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
         <v>2019</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Tex</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Inaugural</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1180,7 +1246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1224,6 +1290,11 @@
           <t>paid_date</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>strengths</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1256,6 +1327,11 @@
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>steady off the tee</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1288,6 +1364,7 @@
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1320,6 +1397,7 @@
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1352,6 +1430,7 @@
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1384,6 +1463,11 @@
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>long drives</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1408,6 +1492,7 @@
           <t>2026-08-20</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>